<commit_message>
Update Richards Physical Architecture.xlsx
</commit_message>
<xml_diff>
--- a/Richards Physical Architecture.xlsx
+++ b/Richards Physical Architecture.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/88f711ca7a7dd18d/Documents/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/88f711ca7a7dd18d/Documents/Git Hub/AIAA-Systems-Engineering-Workshop/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="2" documentId="8_{DD378AB2-C731-40E5-B019-1B596EC618F5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{A06A11C8-8F95-465C-881D-CFCF723909F6}"/>
+  <xr:revisionPtr revIDLastSave="81" documentId="8_{DD378AB2-C731-40E5-B019-1B596EC618F5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{5F8FA727-AFBA-46D6-9A81-B2F9A773A890}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15500" xr2:uid="{71DB06DC-C68B-48CB-8847-6FDAC252FA21}"/>
   </bookViews>
@@ -35,6 +35,92 @@
 </workbook>
 </file>
 
+<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="34" uniqueCount="27">
+  <si>
+    <t>Physical Architecture</t>
+  </si>
+  <si>
+    <t>System-of-system</t>
+  </si>
+  <si>
+    <t>Whole System</t>
+  </si>
+  <si>
+    <t>System</t>
+  </si>
+  <si>
+    <t>Subsystem</t>
+  </si>
+  <si>
+    <t>Element</t>
+  </si>
+  <si>
+    <t>Component</t>
+  </si>
+  <si>
+    <t>Whole Plane</t>
+  </si>
+  <si>
+    <t>Airframe</t>
+  </si>
+  <si>
+    <t>Fuselage</t>
+  </si>
+  <si>
+    <t>Wings</t>
+  </si>
+  <si>
+    <t>Tail</t>
+  </si>
+  <si>
+    <t>Control</t>
+  </si>
+  <si>
+    <t>Identifier</t>
+  </si>
+  <si>
+    <t>Name</t>
+  </si>
+  <si>
+    <t>Spar</t>
+  </si>
+  <si>
+    <t>Interior Mesh</t>
+  </si>
+  <si>
+    <t>Horizontal Stabilizer</t>
+  </si>
+  <si>
+    <t>Vertical Stabilizer</t>
+  </si>
+  <si>
+    <t>Servos</t>
+  </si>
+  <si>
+    <t>Electrical</t>
+  </si>
+  <si>
+    <t>Battery</t>
+  </si>
+  <si>
+    <t>ESC</t>
+  </si>
+  <si>
+    <t>1.1.1</t>
+  </si>
+  <si>
+    <t>1.1.2</t>
+  </si>
+  <si>
+    <t>1.1.3</t>
+  </si>
+  <si>
+    <t>Wing Box</t>
+  </si>
+</sst>
+</file>
+
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <fonts count="1" x14ac:knownFonts="1">
@@ -46,12 +132,18 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="1"/>
+        <bgColor indexed="64"/>
+      </patternFill>
     </fill>
   </fills>
   <borders count="1">
@@ -66,8 +158,12 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -402,9 +498,176 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4C1AF256-8B42-40B1-91C5-D0C8D4ABDE08}">
-  <dimension ref="A1"/>
+  <dimension ref="A1:H23"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
-  <sheetData/>
+  <cols>
+    <col min="1" max="1" width="15.6328125" customWidth="1"/>
+    <col min="2" max="2" width="12" customWidth="1"/>
+    <col min="3" max="3" width="12.1796875" customWidth="1"/>
+    <col min="4" max="4" width="13.90625" customWidth="1"/>
+    <col min="5" max="5" width="13.54296875" customWidth="1"/>
+    <col min="6" max="6" width="3.26953125" style="2" customWidth="1"/>
+    <col min="7" max="7" width="9.1796875" customWidth="1"/>
+    <col min="8" max="8" width="12.1796875" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1"/>
+      <c r="C1" s="1"/>
+      <c r="D1" s="1"/>
+      <c r="E1" s="1"/>
+      <c r="G1" t="s">
+        <v>13</v>
+      </c>
+      <c r="H1" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="2" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A2" t="s">
+        <v>1</v>
+      </c>
+      <c r="B2" t="s">
+        <v>3</v>
+      </c>
+      <c r="C2" t="s">
+        <v>4</v>
+      </c>
+      <c r="D2" t="s">
+        <v>5</v>
+      </c>
+      <c r="E2" t="s">
+        <v>6</v>
+      </c>
+      <c r="G2">
+        <v>0</v>
+      </c>
+      <c r="H2" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="3" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A3" t="s">
+        <v>2</v>
+      </c>
+      <c r="G3">
+        <v>1</v>
+      </c>
+      <c r="H3" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="4" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="B4" t="s">
+        <v>7</v>
+      </c>
+      <c r="G4">
+        <v>1.1000000000000001</v>
+      </c>
+      <c r="H4" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="5" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="C5" t="s">
+        <v>8</v>
+      </c>
+      <c r="G5" t="s">
+        <v>23</v>
+      </c>
+      <c r="H5" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="6" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="D6" t="s">
+        <v>9</v>
+      </c>
+      <c r="G6" t="s">
+        <v>24</v>
+      </c>
+      <c r="H6" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="7" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="E7" t="s">
+        <v>15</v>
+      </c>
+      <c r="G7" t="s">
+        <v>25</v>
+      </c>
+      <c r="H7" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="8" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="E8" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="9" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="E9" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="10" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="D10" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="11" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="E11" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="12" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="D12" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="13" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="E13" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="14" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="E14" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="18" spans="3:4" x14ac:dyDescent="0.35">
+      <c r="C18" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="19" spans="3:4" x14ac:dyDescent="0.35">
+      <c r="D19" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="21" spans="3:4" x14ac:dyDescent="0.35">
+      <c r="C21" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="22" spans="3:4" x14ac:dyDescent="0.35">
+      <c r="D22" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="23" spans="3:4" x14ac:dyDescent="0.35">
+      <c r="D23" t="s">
+        <v>22</v>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A1:E1"/>
+  </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>